<commit_message>
Update workflows to display separately with name matching requirement and add premium HTML report generation
</commit_message>
<xml_diff>
--- a/volunteersync/test/e2e/reports/load_test_report.xlsx
+++ b/volunteersync/test/e2e/reports/load_test_report.xlsx
@@ -20,7 +20,7 @@
     <t>Generated At</t>
   </si>
   <si>
-    <t>23/7/2026, 10:38:59 am</t>
+    <t>25/7/2026, 9:29:17 pm</t>
   </si>
   <si>
     <t>Suite</t>
@@ -148,7 +148,7 @@
     <t>P95 latency measured at 140ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.523Z</t>
+    <t>2026-07-25T15:58:25.558Z</t>
   </si>
   <si>
     <t>Within specifications.</t>
@@ -166,7 +166,7 @@
     <t>P95 latency measured at 160ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.565Z</t>
+    <t>2026-07-25T15:58:25.601Z</t>
   </si>
   <si>
     <t>LND-LOAD-03</t>
@@ -181,7 +181,7 @@
     <t>P95 latency measured at 180ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.573Z</t>
+    <t>2026-07-25T15:58:25.609Z</t>
   </si>
   <si>
     <t>LND-LOAD-04</t>
@@ -193,7 +193,7 @@
     <t>P95 latency measured at 200ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.581Z</t>
+    <t>2026-07-25T15:58:25.617Z</t>
   </si>
   <si>
     <t>LND-LOAD-05</t>
@@ -205,7 +205,7 @@
     <t>P95 latency measured at 220ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.589Z</t>
+    <t>2026-07-25T15:58:25.631Z</t>
   </si>
   <si>
     <t>LND-LOAD-06</t>
@@ -217,7 +217,7 @@
     <t>P95 latency measured at 240ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.598Z</t>
+    <t>2026-07-25T15:58:25.639Z</t>
   </si>
   <si>
     <t>LND-LOAD-07</t>
@@ -229,7 +229,7 @@
     <t>P95 latency measured at 260ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.605Z</t>
+    <t>2026-07-25T15:58:25.646Z</t>
   </si>
   <si>
     <t>LND-LOAD-08</t>
@@ -241,7 +241,7 @@
     <t>P95 latency measured at 280ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.615Z</t>
+    <t>2026-07-25T15:58:25.652Z</t>
   </si>
   <si>
     <t>LND-LOAD-09</t>
@@ -253,7 +253,7 @@
     <t>P95 latency measured at 300ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.624Z</t>
+    <t>2026-07-25T15:58:25.662Z</t>
   </si>
   <si>
     <t>LND-LOAD-10</t>
@@ -265,7 +265,7 @@
     <t>P95 latency measured at 320ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.631Z</t>
+    <t>2026-07-25T15:58:25.672Z</t>
   </si>
   <si>
     <t>LND-LOAD-11</t>
@@ -277,7 +277,7 @@
     <t>P95 latency measured at 340ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.639Z</t>
+    <t>2026-07-25T15:58:25.685Z</t>
   </si>
   <si>
     <t>LND-LOAD-12</t>
@@ -289,7 +289,7 @@
     <t>P95 latency measured at 360ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.649Z</t>
+    <t>2026-07-25T15:58:25.708Z</t>
   </si>
   <si>
     <t>LND-LOAD-13</t>
@@ -301,7 +301,7 @@
     <t>P95 latency measured at 380ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.655Z</t>
+    <t>2026-07-25T15:58:25.718Z</t>
   </si>
   <si>
     <t>LND-LOAD-14</t>
@@ -313,7 +313,7 @@
     <t>P95 latency measured at 400ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.664Z</t>
+    <t>2026-07-25T15:58:25.731Z</t>
   </si>
   <si>
     <t>LND-LOAD-15</t>
@@ -325,7 +325,7 @@
     <t>P95 latency measured at 120ms (0% error rate)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.670Z</t>
+    <t>2026-07-25T15:58:25.737Z</t>
   </si>
   <si>
     <t>LND-LOAD-16</t>
@@ -334,7 +334,7 @@
     <t>Verify Landing screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.678Z</t>
+    <t>2026-07-25T15:58:25.743Z</t>
   </si>
   <si>
     <t>LND-LOAD-17</t>
@@ -343,7 +343,7 @@
     <t>Verify Landing screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.686Z</t>
+    <t>2026-07-25T15:58:25.751Z</t>
   </si>
   <si>
     <t>LND-LOAD-18</t>
@@ -352,7 +352,7 @@
     <t>Verify Landing screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.693Z</t>
+    <t>2026-07-25T15:58:25.756Z</t>
   </si>
   <si>
     <t>LND-LOAD-19</t>
@@ -361,7 +361,7 @@
     <t>Verify Landing screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.702Z</t>
+    <t>2026-07-25T15:58:25.763Z</t>
   </si>
   <si>
     <t>LND-LOAD-20</t>
@@ -370,7 +370,7 @@
     <t>Verify Landing screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.709Z</t>
+    <t>2026-07-25T15:58:25.770Z</t>
   </si>
   <si>
     <t>LND-LOAD-21</t>
@@ -379,7 +379,7 @@
     <t>Verify Landing screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.716Z</t>
+    <t>2026-07-25T15:58:25.776Z</t>
   </si>
   <si>
     <t>LND-LOAD-22</t>
@@ -388,7 +388,7 @@
     <t>Verify Landing screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.725Z</t>
+    <t>2026-07-25T15:58:25.782Z</t>
   </si>
   <si>
     <t>LND-LOAD-23</t>
@@ -397,7 +397,7 @@
     <t>Verify Landing screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.733Z</t>
+    <t>2026-07-25T15:58:25.789Z</t>
   </si>
   <si>
     <t>LND-LOAD-24</t>
@@ -406,7 +406,7 @@
     <t>Verify Landing screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.741Z</t>
+    <t>2026-07-25T15:58:25.798Z</t>
   </si>
   <si>
     <t>LND-LOAD-25</t>
@@ -415,7 +415,7 @@
     <t>Verify Landing screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.750Z</t>
+    <t>2026-07-25T15:58:25.808Z</t>
   </si>
   <si>
     <t>LND-LOAD-26</t>
@@ -424,7 +424,7 @@
     <t>Verify Landing screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.761Z</t>
+    <t>2026-07-25T15:58:25.816Z</t>
   </si>
   <si>
     <t>LND-LOAD-27</t>
@@ -433,7 +433,7 @@
     <t>Verify Landing screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.770Z</t>
+    <t>2026-07-25T15:58:25.824Z</t>
   </si>
   <si>
     <t>LND-LOAD-28</t>
@@ -442,7 +442,7 @@
     <t>Verify Landing screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.779Z</t>
+    <t>2026-07-25T15:58:25.834Z</t>
   </si>
   <si>
     <t>LND-LOAD-29</t>
@@ -451,7 +451,7 @@
     <t>Verify Landing screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.790Z</t>
+    <t>2026-07-25T15:58:25.842Z</t>
   </si>
   <si>
     <t>LND-LOAD-30</t>
@@ -460,7 +460,7 @@
     <t>Verify Landing screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.799Z</t>
+    <t>2026-07-25T15:58:25.850Z</t>
   </si>
   <si>
     <t>LND-LOAD-31</t>
@@ -469,7 +469,7 @@
     <t>Verify Landing screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.808Z</t>
+    <t>2026-07-25T15:58:25.859Z</t>
   </si>
   <si>
     <t>LND-LOAD-32</t>
@@ -478,7 +478,7 @@
     <t>Verify Landing screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.820Z</t>
+    <t>2026-07-25T15:58:25.871Z</t>
   </si>
   <si>
     <t>LND-LOAD-33</t>
@@ -487,7 +487,7 @@
     <t>Verify Landing screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.830Z</t>
+    <t>2026-07-25T15:58:25.880Z</t>
   </si>
   <si>
     <t>LND-LOAD-34</t>
@@ -496,7 +496,7 @@
     <t>Verify Landing screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.838Z</t>
+    <t>2026-07-25T15:58:25.887Z</t>
   </si>
   <si>
     <t>LND-LOAD-35</t>
@@ -505,7 +505,7 @@
     <t>Verify Landing screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.847Z</t>
+    <t>2026-07-25T15:58:25.895Z</t>
   </si>
   <si>
     <t>LND-LOAD-36</t>
@@ -514,7 +514,7 @@
     <t>Verify Landing screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.855Z</t>
+    <t>2026-07-25T15:58:25.902Z</t>
   </si>
   <si>
     <t>LOG-LOAD-01</t>
@@ -523,7 +523,7 @@
     <t>Verify Login screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.864Z</t>
+    <t>2026-07-25T15:58:25.912Z</t>
   </si>
   <si>
     <t>LOG-LOAD-02</t>
@@ -532,7 +532,7 @@
     <t>Verify Login screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.872Z</t>
+    <t>2026-07-25T15:58:25.920Z</t>
   </si>
   <si>
     <t>LOG-LOAD-03</t>
@@ -541,7 +541,7 @@
     <t>Verify Login screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.882Z</t>
+    <t>2026-07-25T15:58:25.932Z</t>
   </si>
   <si>
     <t>LOG-LOAD-04</t>
@@ -550,7 +550,7 @@
     <t>Verify Login screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.891Z</t>
+    <t>2026-07-25T15:58:25.945Z</t>
   </si>
   <si>
     <t>LOG-LOAD-05</t>
@@ -559,7 +559,7 @@
     <t>Verify Login screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.901Z</t>
+    <t>2026-07-25T15:58:25.955Z</t>
   </si>
   <si>
     <t>LOG-LOAD-06</t>
@@ -568,7 +568,7 @@
     <t>Verify Login screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.916Z</t>
+    <t>2026-07-25T15:58:25.968Z</t>
   </si>
   <si>
     <t>LOG-LOAD-07</t>
@@ -577,7 +577,7 @@
     <t>Verify Login screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.925Z</t>
+    <t>2026-07-25T15:58:25.976Z</t>
   </si>
   <si>
     <t>LOG-LOAD-08</t>
@@ -586,7 +586,7 @@
     <t>Verify Login screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.936Z</t>
+    <t>2026-07-25T15:58:25.987Z</t>
   </si>
   <si>
     <t>LOG-LOAD-09</t>
@@ -595,7 +595,7 @@
     <t>Verify Login screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.945Z</t>
+    <t>2026-07-25T15:58:25.999Z</t>
   </si>
   <si>
     <t>LOG-LOAD-10</t>
@@ -604,7 +604,7 @@
     <t>Verify Login screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.953Z</t>
+    <t>2026-07-25T15:58:26.009Z</t>
   </si>
   <si>
     <t>LOG-LOAD-11</t>
@@ -613,7 +613,7 @@
     <t>Verify Login screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.964Z</t>
+    <t>2026-07-25T15:58:26.018Z</t>
   </si>
   <si>
     <t>LOG-LOAD-12</t>
@@ -622,7 +622,7 @@
     <t>Verify Login screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.974Z</t>
+    <t>2026-07-25T15:58:26.029Z</t>
   </si>
   <si>
     <t>LOG-LOAD-13</t>
@@ -631,7 +631,7 @@
     <t>Verify Login screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.984Z</t>
+    <t>2026-07-25T15:58:26.038Z</t>
   </si>
   <si>
     <t>LOG-LOAD-14</t>
@@ -640,7 +640,7 @@
     <t>Verify Login screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:45.993Z</t>
+    <t>2026-07-25T15:58:26.048Z</t>
   </si>
   <si>
     <t>LOG-LOAD-15</t>
@@ -649,7 +649,7 @@
     <t>Verify Login screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.004Z</t>
+    <t>2026-07-25T15:58:26.057Z</t>
   </si>
   <si>
     <t>LOG-LOAD-16</t>
@@ -658,7 +658,7 @@
     <t>Verify Login screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.014Z</t>
+    <t>2026-07-25T15:58:26.067Z</t>
   </si>
   <si>
     <t>LOG-LOAD-17</t>
@@ -667,7 +667,7 @@
     <t>Verify Login screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.025Z</t>
+    <t>2026-07-25T15:58:26.078Z</t>
   </si>
   <si>
     <t>LOG-LOAD-18</t>
@@ -676,7 +676,7 @@
     <t>Verify Login screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.035Z</t>
+    <t>2026-07-25T15:58:26.088Z</t>
   </si>
   <si>
     <t>LOG-LOAD-19</t>
@@ -685,7 +685,7 @@
     <t>Verify Login screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.046Z</t>
+    <t>2026-07-25T15:58:26.105Z</t>
   </si>
   <si>
     <t>LOG-LOAD-20</t>
@@ -694,7 +694,7 @@
     <t>Verify Login screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.056Z</t>
+    <t>2026-07-25T15:58:26.115Z</t>
   </si>
   <si>
     <t>LOG-LOAD-21</t>
@@ -703,7 +703,7 @@
     <t>Verify Login screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.067Z</t>
+    <t>2026-07-25T15:58:26.128Z</t>
   </si>
   <si>
     <t>LOG-LOAD-22</t>
@@ -712,7 +712,7 @@
     <t>Verify Login screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.079Z</t>
+    <t>2026-07-25T15:58:26.144Z</t>
   </si>
   <si>
     <t>LOG-LOAD-23</t>
@@ -721,7 +721,7 @@
     <t>Verify Login screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.090Z</t>
+    <t>2026-07-25T15:58:26.157Z</t>
   </si>
   <si>
     <t>LOG-LOAD-24</t>
@@ -730,7 +730,7 @@
     <t>Verify Login screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.102Z</t>
+    <t>2026-07-25T15:58:26.177Z</t>
   </si>
   <si>
     <t>LOG-LOAD-25</t>
@@ -739,7 +739,7 @@
     <t>Verify Login screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.113Z</t>
+    <t>2026-07-25T15:58:26.191Z</t>
   </si>
   <si>
     <t>LOG-LOAD-26</t>
@@ -748,7 +748,7 @@
     <t>Verify Login screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.125Z</t>
+    <t>2026-07-25T15:58:26.204Z</t>
   </si>
   <si>
     <t>LOG-LOAD-27</t>
@@ -757,7 +757,7 @@
     <t>Verify Login screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.138Z</t>
+    <t>2026-07-25T15:58:26.214Z</t>
   </si>
   <si>
     <t>LOG-LOAD-28</t>
@@ -766,7 +766,7 @@
     <t>Verify Login screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.150Z</t>
+    <t>2026-07-25T15:58:26.229Z</t>
   </si>
   <si>
     <t>LOG-LOAD-29</t>
@@ -775,7 +775,7 @@
     <t>Verify Login screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.161Z</t>
+    <t>2026-07-25T15:58:26.243Z</t>
   </si>
   <si>
     <t>LOG-LOAD-30</t>
@@ -784,7 +784,7 @@
     <t>Verify Login screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.174Z</t>
+    <t>2026-07-25T15:58:26.261Z</t>
   </si>
   <si>
     <t>LOG-LOAD-31</t>
@@ -793,7 +793,7 @@
     <t>Verify Login screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.185Z</t>
+    <t>2026-07-25T15:58:26.276Z</t>
   </si>
   <si>
     <t>LOG-LOAD-32</t>
@@ -802,7 +802,7 @@
     <t>Verify Login screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.199Z</t>
+    <t>2026-07-25T15:58:26.322Z</t>
   </si>
   <si>
     <t>LOG-LOAD-33</t>
@@ -811,7 +811,7 @@
     <t>Verify Login screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.213Z</t>
+    <t>2026-07-25T15:58:26.336Z</t>
   </si>
   <si>
     <t>LOG-LOAD-34</t>
@@ -820,7 +820,7 @@
     <t>Verify Login screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.227Z</t>
+    <t>2026-07-25T15:58:26.350Z</t>
   </si>
   <si>
     <t>LOG-LOAD-35</t>
@@ -829,7 +829,7 @@
     <t>Verify Login screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.239Z</t>
+    <t>2026-07-25T15:58:26.365Z</t>
   </si>
   <si>
     <t>LOG-LOAD-36</t>
@@ -838,7 +838,7 @@
     <t>Verify Login screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.253Z</t>
+    <t>2026-07-25T15:58:26.381Z</t>
   </si>
   <si>
     <t>REG-LOAD-01</t>
@@ -847,7 +847,7 @@
     <t>Verify Register screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.264Z</t>
+    <t>2026-07-25T15:58:26.395Z</t>
   </si>
   <si>
     <t>REG-LOAD-02</t>
@@ -856,7 +856,7 @@
     <t>Verify Register screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.280Z</t>
+    <t>2026-07-25T15:58:26.415Z</t>
   </si>
   <si>
     <t>REG-LOAD-03</t>
@@ -865,7 +865,7 @@
     <t>Verify Register screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.296Z</t>
+    <t>2026-07-25T15:58:26.432Z</t>
   </si>
   <si>
     <t>REG-LOAD-04</t>
@@ -874,7 +874,7 @@
     <t>Verify Register screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.310Z</t>
+    <t>2026-07-25T15:58:26.452Z</t>
   </si>
   <si>
     <t>REG-LOAD-05</t>
@@ -883,7 +883,7 @@
     <t>Verify Register screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.323Z</t>
+    <t>2026-07-25T15:58:26.470Z</t>
   </si>
   <si>
     <t>REG-LOAD-06</t>
@@ -892,7 +892,7 @@
     <t>Verify Register screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.337Z</t>
+    <t>2026-07-25T15:58:26.484Z</t>
   </si>
   <si>
     <t>REG-LOAD-07</t>
@@ -901,7 +901,7 @@
     <t>Verify Register screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.354Z</t>
+    <t>2026-07-25T15:58:26.498Z</t>
   </si>
   <si>
     <t>REG-LOAD-08</t>
@@ -910,7 +910,7 @@
     <t>Verify Register screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.371Z</t>
+    <t>2026-07-25T15:58:26.513Z</t>
   </si>
   <si>
     <t>REG-LOAD-09</t>
@@ -919,7 +919,7 @@
     <t>Verify Register screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.385Z</t>
+    <t>2026-07-25T15:58:26.524Z</t>
   </si>
   <si>
     <t>REG-LOAD-10</t>
@@ -928,7 +928,7 @@
     <t>Verify Register screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.398Z</t>
+    <t>2026-07-25T15:58:26.543Z</t>
   </si>
   <si>
     <t>REG-LOAD-11</t>
@@ -937,7 +937,7 @@
     <t>Verify Register screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.410Z</t>
+    <t>2026-07-25T15:58:26.558Z</t>
   </si>
   <si>
     <t>REG-LOAD-12</t>
@@ -946,7 +946,7 @@
     <t>Verify Register screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.424Z</t>
+    <t>2026-07-25T15:58:26.576Z</t>
   </si>
   <si>
     <t>REG-LOAD-13</t>
@@ -955,7 +955,7 @@
     <t>Verify Register screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.452Z</t>
+    <t>2026-07-25T15:58:26.589Z</t>
   </si>
   <si>
     <t>REG-LOAD-14</t>
@@ -964,7 +964,7 @@
     <t>Verify Register screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.481Z</t>
+    <t>2026-07-25T15:58:26.604Z</t>
   </si>
   <si>
     <t>REG-LOAD-15</t>
@@ -973,7 +973,7 @@
     <t>Verify Register screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.496Z</t>
+    <t>2026-07-25T15:58:26.616Z</t>
   </si>
   <si>
     <t>REG-LOAD-16</t>
@@ -982,7 +982,7 @@
     <t>Verify Register screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.512Z</t>
+    <t>2026-07-25T15:58:26.629Z</t>
   </si>
   <si>
     <t>REG-LOAD-17</t>
@@ -991,7 +991,7 @@
     <t>Verify Register screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.529Z</t>
+    <t>2026-07-25T15:58:26.643Z</t>
   </si>
   <si>
     <t>REG-LOAD-18</t>
@@ -1000,7 +1000,7 @@
     <t>Verify Register screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.547Z</t>
+    <t>2026-07-25T15:58:26.656Z</t>
   </si>
   <si>
     <t>REG-LOAD-19</t>
@@ -1009,7 +1009,7 @@
     <t>Verify Register screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.564Z</t>
+    <t>2026-07-25T15:58:26.672Z</t>
   </si>
   <si>
     <t>REG-LOAD-20</t>
@@ -1018,7 +1018,7 @@
     <t>Verify Register screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.580Z</t>
+    <t>2026-07-25T15:58:26.685Z</t>
   </si>
   <si>
     <t>REG-LOAD-21</t>
@@ -1027,7 +1027,7 @@
     <t>Verify Register screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.595Z</t>
+    <t>2026-07-25T15:58:26.703Z</t>
   </si>
   <si>
     <t>REG-LOAD-22</t>
@@ -1036,7 +1036,7 @@
     <t>Verify Register screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.609Z</t>
+    <t>2026-07-25T15:58:26.718Z</t>
   </si>
   <si>
     <t>REG-LOAD-23</t>
@@ -1045,7 +1045,7 @@
     <t>Verify Register screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.624Z</t>
+    <t>2026-07-25T15:58:26.738Z</t>
   </si>
   <si>
     <t>REG-LOAD-24</t>
@@ -1054,7 +1054,7 @@
     <t>Verify Register screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.641Z</t>
+    <t>2026-07-25T15:58:26.754Z</t>
   </si>
   <si>
     <t>REG-LOAD-25</t>
@@ -1063,7 +1063,7 @@
     <t>Verify Register screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.657Z</t>
+    <t>2026-07-25T15:58:26.771Z</t>
   </si>
   <si>
     <t>REG-LOAD-26</t>
@@ -1072,7 +1072,7 @@
     <t>Verify Register screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.673Z</t>
+    <t>2026-07-25T15:58:26.786Z</t>
   </si>
   <si>
     <t>REG-LOAD-27</t>
@@ -1081,7 +1081,7 @@
     <t>Verify Register screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.689Z</t>
+    <t>2026-07-25T15:58:26.804Z</t>
   </si>
   <si>
     <t>REG-LOAD-28</t>
@@ -1090,7 +1090,7 @@
     <t>Verify Register screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.703Z</t>
+    <t>2026-07-25T15:58:26.819Z</t>
   </si>
   <si>
     <t>REG-LOAD-29</t>
@@ -1099,7 +1099,7 @@
     <t>Verify Register screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.721Z</t>
+    <t>2026-07-25T15:58:26.864Z</t>
   </si>
   <si>
     <t>REG-LOAD-30</t>
@@ -1108,7 +1108,7 @@
     <t>Verify Register screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.738Z</t>
+    <t>2026-07-25T15:58:26.881Z</t>
   </si>
   <si>
     <t>REG-LOAD-31</t>
@@ -1117,7 +1117,7 @@
     <t>Verify Register screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.754Z</t>
+    <t>2026-07-25T15:58:26.896Z</t>
   </si>
   <si>
     <t>REG-LOAD-32</t>
@@ -1126,7 +1126,7 @@
     <t>Verify Register screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.774Z</t>
+    <t>2026-07-25T15:58:26.912Z</t>
   </si>
   <si>
     <t>REG-LOAD-33</t>
@@ -1135,7 +1135,7 @@
     <t>Verify Register screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.790Z</t>
+    <t>2026-07-25T15:58:26.925Z</t>
   </si>
   <si>
     <t>REG-LOAD-34</t>
@@ -1144,7 +1144,7 @@
     <t>Verify Register screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.805Z</t>
+    <t>2026-07-25T15:58:26.940Z</t>
   </si>
   <si>
     <t>REG-LOAD-35</t>
@@ -1153,7 +1153,7 @@
     <t>Verify Register screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.825Z</t>
+    <t>2026-07-25T15:58:26.958Z</t>
   </si>
   <si>
     <t>REG-LOAD-36</t>
@@ -1162,7 +1162,7 @@
     <t>Verify Register screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.843Z</t>
+    <t>2026-07-25T15:58:26.974Z</t>
   </si>
   <si>
     <t>FP-LOAD-01</t>
@@ -1171,7 +1171,7 @@
     <t>Verify ForgotPassword screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.861Z</t>
+    <t>2026-07-25T15:58:26.990Z</t>
   </si>
   <si>
     <t>FP-LOAD-02</t>
@@ -1180,7 +1180,7 @@
     <t>Verify ForgotPassword screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.880Z</t>
+    <t>2026-07-25T15:58:27.006Z</t>
   </si>
   <si>
     <t>FP-LOAD-03</t>
@@ -1189,7 +1189,7 @@
     <t>Verify ForgotPassword screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.901Z</t>
+    <t>2026-07-25T15:58:27.023Z</t>
   </si>
   <si>
     <t>FP-LOAD-04</t>
@@ -1198,7 +1198,7 @@
     <t>Verify ForgotPassword screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.926Z</t>
+    <t>2026-07-25T15:58:27.045Z</t>
   </si>
   <si>
     <t>FP-LOAD-05</t>
@@ -1207,7 +1207,7 @@
     <t>Verify ForgotPassword screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.952Z</t>
+    <t>2026-07-25T15:58:27.094Z</t>
   </si>
   <si>
     <t>FP-LOAD-06</t>
@@ -1216,7 +1216,7 @@
     <t>Verify ForgotPassword screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.970Z</t>
+    <t>2026-07-25T15:58:27.194Z</t>
   </si>
   <si>
     <t>FP-LOAD-07</t>
@@ -1225,7 +1225,7 @@
     <t>Verify ForgotPassword screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:46.987Z</t>
+    <t>2026-07-25T15:58:27.302Z</t>
   </si>
   <si>
     <t>FP-LOAD-08</t>
@@ -1234,7 +1234,7 @@
     <t>Verify ForgotPassword screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.004Z</t>
+    <t>2026-07-25T15:58:27.390Z</t>
   </si>
   <si>
     <t>FP-LOAD-09</t>
@@ -1243,7 +1243,7 @@
     <t>Verify ForgotPassword screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.050Z</t>
+    <t>2026-07-25T15:58:27.478Z</t>
   </si>
   <si>
     <t>FP-LOAD-10</t>
@@ -1252,7 +1252,7 @@
     <t>Verify ForgotPassword screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.075Z</t>
+    <t>2026-07-25T15:58:27.567Z</t>
   </si>
   <si>
     <t>FP-LOAD-11</t>
@@ -1261,7 +1261,7 @@
     <t>Verify ForgotPassword screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.092Z</t>
+    <t>2026-07-25T15:58:27.646Z</t>
   </si>
   <si>
     <t>FP-LOAD-12</t>
@@ -1270,7 +1270,7 @@
     <t>Verify ForgotPassword screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.111Z</t>
+    <t>2026-07-25T15:58:27.732Z</t>
   </si>
   <si>
     <t>FP-LOAD-13</t>
@@ -1279,7 +1279,7 @@
     <t>Verify ForgotPassword screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.128Z</t>
+    <t>2026-07-25T15:58:27.808Z</t>
   </si>
   <si>
     <t>FP-LOAD-14</t>
@@ -1288,7 +1288,7 @@
     <t>Verify ForgotPassword screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.146Z</t>
+    <t>2026-07-25T15:58:27.878Z</t>
   </si>
   <si>
     <t>FP-LOAD-15</t>
@@ -1297,7 +1297,7 @@
     <t>Verify ForgotPassword screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.164Z</t>
+    <t>2026-07-25T15:58:27.949Z</t>
   </si>
   <si>
     <t>FP-LOAD-16</t>
@@ -1306,7 +1306,7 @@
     <t>Verify ForgotPassword screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.182Z</t>
+    <t>2026-07-25T15:58:28.034Z</t>
   </si>
   <si>
     <t>FP-LOAD-17</t>
@@ -1315,7 +1315,7 @@
     <t>Verify ForgotPassword screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.215Z</t>
+    <t>2026-07-25T15:58:28.147Z</t>
   </si>
   <si>
     <t>FP-LOAD-18</t>
@@ -1324,7 +1324,7 @@
     <t>Verify ForgotPassword screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.237Z</t>
+    <t>2026-07-25T15:58:28.261Z</t>
   </si>
   <si>
     <t>FP-LOAD-19</t>
@@ -1333,7 +1333,7 @@
     <t>Verify ForgotPassword screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.259Z</t>
+    <t>2026-07-25T15:58:28.348Z</t>
   </si>
   <si>
     <t>FP-LOAD-20</t>
@@ -1342,7 +1342,7 @@
     <t>Verify ForgotPassword screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.286Z</t>
+    <t>2026-07-25T15:58:28.444Z</t>
   </si>
   <si>
     <t>FP-LOAD-21</t>
@@ -1351,7 +1351,7 @@
     <t>Verify ForgotPassword screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.314Z</t>
+    <t>2026-07-25T15:58:28.528Z</t>
   </si>
   <si>
     <t>FP-LOAD-22</t>
@@ -1360,7 +1360,7 @@
     <t>Verify ForgotPassword screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.356Z</t>
+    <t>2026-07-25T15:58:28.611Z</t>
   </si>
   <si>
     <t>FP-LOAD-23</t>
@@ -1369,7 +1369,7 @@
     <t>Verify ForgotPassword screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.377Z</t>
+    <t>2026-07-25T15:58:28.731Z</t>
   </si>
   <si>
     <t>FP-LOAD-24</t>
@@ -1378,7 +1378,7 @@
     <t>Verify ForgotPassword screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.398Z</t>
+    <t>2026-07-25T15:58:28.922Z</t>
   </si>
   <si>
     <t>FP-LOAD-25</t>
@@ -1387,7 +1387,7 @@
     <t>Verify ForgotPassword screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.420Z</t>
+    <t>2026-07-25T15:58:29.147Z</t>
   </si>
   <si>
     <t>FP-LOAD-26</t>
@@ -1396,7 +1396,7 @@
     <t>Verify ForgotPassword screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.442Z</t>
+    <t>2026-07-25T15:58:29.305Z</t>
   </si>
   <si>
     <t>FP-LOAD-27</t>
@@ -1405,7 +1405,7 @@
     <t>Verify ForgotPassword screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.470Z</t>
+    <t>2026-07-25T15:58:29.416Z</t>
   </si>
   <si>
     <t>FP-LOAD-28</t>
@@ -1414,7 +1414,7 @@
     <t>Verify ForgotPassword screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.505Z</t>
+    <t>2026-07-25T15:58:29.525Z</t>
   </si>
   <si>
     <t>FP-LOAD-29</t>
@@ -1423,7 +1423,7 @@
     <t>Verify ForgotPassword screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.551Z</t>
+    <t>2026-07-25T15:58:29.642Z</t>
   </si>
   <si>
     <t>FP-LOAD-30</t>
@@ -1432,7 +1432,7 @@
     <t>Verify ForgotPassword screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.596Z</t>
+    <t>2026-07-25T15:58:29.743Z</t>
   </si>
   <si>
     <t>FP-LOAD-31</t>
@@ -1441,7 +1441,7 @@
     <t>Verify ForgotPassword screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.625Z</t>
+    <t>2026-07-25T15:58:29.837Z</t>
   </si>
   <si>
     <t>FP-LOAD-32</t>
@@ -1450,7 +1450,7 @@
     <t>Verify ForgotPassword screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.649Z</t>
+    <t>2026-07-25T15:58:29.932Z</t>
   </si>
   <si>
     <t>FP-LOAD-33</t>
@@ -1459,7 +1459,7 @@
     <t>Verify ForgotPassword screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.672Z</t>
+    <t>2026-07-25T15:58:30.028Z</t>
   </si>
   <si>
     <t>FP-LOAD-34</t>
@@ -1468,7 +1468,7 @@
     <t>Verify ForgotPassword screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.706Z</t>
+    <t>2026-07-25T15:58:30.139Z</t>
   </si>
   <si>
     <t>FP-LOAD-35</t>
@@ -1477,7 +1477,7 @@
     <t>Verify ForgotPassword screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.744Z</t>
+    <t>2026-07-25T15:58:30.248Z</t>
   </si>
   <si>
     <t>FP-LOAD-36</t>
@@ -1486,7 +1486,7 @@
     <t>Verify ForgotPassword screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.797Z</t>
+    <t>2026-07-25T15:58:30.347Z</t>
   </si>
   <si>
     <t>DASH-LOAD-01</t>
@@ -1495,7 +1495,7 @@
     <t>Verify Dashboard screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.831Z</t>
+    <t>2026-07-25T15:58:30.441Z</t>
   </si>
   <si>
     <t>DASH-LOAD-02</t>
@@ -1504,7 +1504,7 @@
     <t>Verify Dashboard screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.856Z</t>
+    <t>2026-07-25T15:58:30.537Z</t>
   </si>
   <si>
     <t>DASH-LOAD-03</t>
@@ -1513,7 +1513,7 @@
     <t>Verify Dashboard screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.876Z</t>
+    <t>2026-07-25T15:58:30.632Z</t>
   </si>
   <si>
     <t>DASH-LOAD-04</t>
@@ -1522,7 +1522,7 @@
     <t>Verify Dashboard screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.910Z</t>
+    <t>2026-07-25T15:58:30.765Z</t>
   </si>
   <si>
     <t>DASH-LOAD-05</t>
@@ -1531,7 +1531,7 @@
     <t>Verify Dashboard screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.963Z</t>
+    <t>2026-07-25T15:58:30.865Z</t>
   </si>
   <si>
     <t>DASH-LOAD-06</t>
@@ -1540,7 +1540,7 @@
     <t>Verify Dashboard screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:47.990Z</t>
+    <t>2026-07-25T15:58:30.974Z</t>
   </si>
   <si>
     <t>DASH-LOAD-07</t>
@@ -1549,7 +1549,7 @@
     <t>Verify Dashboard screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.040Z</t>
+    <t>2026-07-25T15:58:31.097Z</t>
   </si>
   <si>
     <t>DASH-LOAD-08</t>
@@ -1569,7 +1569,7 @@
     <t>Query latency spiked to 3200ms due to database locks</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.070Z</t>
+    <t>2026-07-25T15:58:31.204Z</t>
   </si>
   <si>
     <t>Performance threshold breached.</t>
@@ -1581,7 +1581,7 @@
     <t>Verify Dashboard screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.139Z</t>
+    <t>2026-07-25T15:58:31.308Z</t>
   </si>
   <si>
     <t>DASH-LOAD-10</t>
@@ -1590,7 +1590,7 @@
     <t>Verify Dashboard screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.203Z</t>
+    <t>2026-07-25T15:58:31.397Z</t>
   </si>
   <si>
     <t>DASH-LOAD-11</t>
@@ -1599,7 +1599,7 @@
     <t>Verify Dashboard screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.263Z</t>
+    <t>2026-07-25T15:58:31.509Z</t>
   </si>
   <si>
     <t>DASH-LOAD-12</t>
@@ -1608,7 +1608,7 @@
     <t>Verify Dashboard screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.317Z</t>
+    <t>2026-07-25T15:58:31.583Z</t>
   </si>
   <si>
     <t>DASH-LOAD-13</t>
@@ -1617,7 +1617,7 @@
     <t>Verify Dashboard screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.369Z</t>
+    <t>2026-07-25T15:58:31.678Z</t>
   </si>
   <si>
     <t>DASH-LOAD-14</t>
@@ -1626,7 +1626,7 @@
     <t>Verify Dashboard screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.432Z</t>
+    <t>2026-07-25T15:58:31.775Z</t>
   </si>
   <si>
     <t>DASH-LOAD-15</t>
@@ -1635,7 +1635,7 @@
     <t>Verify Dashboard screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.482Z</t>
+    <t>2026-07-25T15:58:31.853Z</t>
   </si>
   <si>
     <t>DASH-LOAD-16</t>
@@ -1644,7 +1644,7 @@
     <t>Verify Dashboard screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.542Z</t>
+    <t>2026-07-25T15:58:32.037Z</t>
   </si>
   <si>
     <t>DASH-LOAD-17</t>
@@ -1653,7 +1653,7 @@
     <t>Verify Dashboard screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.591Z</t>
+    <t>2026-07-25T15:58:32.155Z</t>
   </si>
   <si>
     <t>DASH-LOAD-18</t>
@@ -1662,7 +1662,7 @@
     <t>Verify Dashboard screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.651Z</t>
+    <t>2026-07-25T15:58:32.289Z</t>
   </si>
   <si>
     <t>DASH-LOAD-19</t>
@@ -1671,7 +1671,7 @@
     <t>Verify Dashboard screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.702Z</t>
+    <t>2026-07-25T15:58:32.398Z</t>
   </si>
   <si>
     <t>DASH-LOAD-20</t>
@@ -1680,7 +1680,7 @@
     <t>Verify Dashboard screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.754Z</t>
+    <t>2026-07-25T15:58:32.528Z</t>
   </si>
   <si>
     <t>DASH-LOAD-21</t>
@@ -1689,7 +1689,7 @@
     <t>Verify Dashboard screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.804Z</t>
+    <t>2026-07-25T15:58:32.617Z</t>
   </si>
   <si>
     <t>DASH-LOAD-22</t>
@@ -1698,7 +1698,7 @@
     <t>Verify Dashboard screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.860Z</t>
+    <t>2026-07-25T15:58:32.739Z</t>
   </si>
   <si>
     <t>DASH-LOAD-23</t>
@@ -1707,7 +1707,7 @@
     <t>Verify Dashboard screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.916Z</t>
+    <t>2026-07-25T15:58:32.856Z</t>
   </si>
   <si>
     <t>DASH-LOAD-24</t>
@@ -1716,7 +1716,7 @@
     <t>Verify Dashboard screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:48.979Z</t>
+    <t>2026-07-25T15:58:32.974Z</t>
   </si>
   <si>
     <t>DASH-LOAD-25</t>
@@ -1725,7 +1725,7 @@
     <t>Verify Dashboard screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.028Z</t>
+    <t>2026-07-25T15:58:33.071Z</t>
   </si>
   <si>
     <t>DASH-LOAD-26</t>
@@ -1734,7 +1734,7 @@
     <t>Verify Dashboard screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.087Z</t>
+    <t>2026-07-25T15:58:33.187Z</t>
   </si>
   <si>
     <t>DASH-LOAD-27</t>
@@ -1743,7 +1743,7 @@
     <t>Verify Dashboard screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.141Z</t>
+    <t>2026-07-25T15:58:33.305Z</t>
   </si>
   <si>
     <t>DASH-LOAD-28</t>
@@ -1752,7 +1752,7 @@
     <t>Verify Dashboard screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.200Z</t>
+    <t>2026-07-25T15:58:33.417Z</t>
   </si>
   <si>
     <t>DASH-LOAD-29</t>
@@ -1761,7 +1761,7 @@
     <t>Verify Dashboard screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.249Z</t>
+    <t>2026-07-25T15:58:33.528Z</t>
   </si>
   <si>
     <t>DASH-LOAD-30</t>
@@ -1770,7 +1770,7 @@
     <t>Verify Dashboard screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.302Z</t>
+    <t>2026-07-25T15:58:33.642Z</t>
   </si>
   <si>
     <t>DASH-LOAD-31</t>
@@ -1779,7 +1779,7 @@
     <t>Verify Dashboard screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.356Z</t>
+    <t>2026-07-25T15:58:33.752Z</t>
   </si>
   <si>
     <t>DASH-LOAD-32</t>
@@ -1788,7 +1788,7 @@
     <t>Verify Dashboard screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.410Z</t>
+    <t>2026-07-25T15:58:33.876Z</t>
   </si>
   <si>
     <t>DASH-LOAD-33</t>
@@ -1797,7 +1797,7 @@
     <t>Verify Dashboard screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.471Z</t>
+    <t>2026-07-25T15:58:33.970Z</t>
   </si>
   <si>
     <t>DASH-LOAD-34</t>
@@ -1806,7 +1806,7 @@
     <t>Verify Dashboard screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.521Z</t>
+    <t>2026-07-25T15:58:34.107Z</t>
   </si>
   <si>
     <t>DASH-LOAD-35</t>
@@ -1815,7 +1815,7 @@
     <t>Verify Dashboard screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.575Z</t>
+    <t>2026-07-25T15:58:34.213Z</t>
   </si>
   <si>
     <t>DASH-LOAD-36</t>
@@ -1824,7 +1824,7 @@
     <t>Verify Dashboard screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.633Z</t>
+    <t>2026-07-25T15:58:34.296Z</t>
   </si>
   <si>
     <t>VOL-LOAD-01</t>
@@ -1833,7 +1833,7 @@
     <t>Verify Volunteers screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.716Z</t>
+    <t>2026-07-25T15:58:34.381Z</t>
   </si>
   <si>
     <t>VOL-LOAD-02</t>
@@ -1842,7 +1842,7 @@
     <t>Verify Volunteers screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.795Z</t>
+    <t>2026-07-25T15:58:34.493Z</t>
   </si>
   <si>
     <t>VOL-LOAD-03</t>
@@ -1851,7 +1851,7 @@
     <t>Verify Volunteers screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.869Z</t>
+    <t>2026-07-25T15:58:34.604Z</t>
   </si>
   <si>
     <t>VOL-LOAD-04</t>
@@ -1860,7 +1860,7 @@
     <t>Verify Volunteers screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.915Z</t>
+    <t>2026-07-25T15:58:34.679Z</t>
   </si>
   <si>
     <t>VOL-LOAD-05</t>
@@ -1869,7 +1869,7 @@
     <t>Verify Volunteers screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.949Z</t>
+    <t>2026-07-25T15:58:34.758Z</t>
   </si>
   <si>
     <t>VOL-LOAD-06</t>
@@ -1878,7 +1878,7 @@
     <t>Verify Volunteers screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:49.973Z</t>
+    <t>2026-07-25T15:58:34.871Z</t>
   </si>
   <si>
     <t>VOL-LOAD-07</t>
@@ -1887,7 +1887,7 @@
     <t>Verify Volunteers screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.000Z</t>
+    <t>2026-07-25T15:58:35.005Z</t>
   </si>
   <si>
     <t>VOL-LOAD-08</t>
@@ -1896,7 +1896,7 @@
     <t>Verify Volunteers screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.024Z</t>
+    <t>2026-07-25T15:58:35.140Z</t>
   </si>
   <si>
     <t>VOL-LOAD-09</t>
@@ -1905,7 +1905,7 @@
     <t>Verify Volunteers screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.055Z</t>
+    <t>2026-07-25T15:58:35.290Z</t>
   </si>
   <si>
     <t>VOL-LOAD-10</t>
@@ -1914,7 +1914,7 @@
     <t>Verify Volunteers screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.085Z</t>
+    <t>2026-07-25T15:58:35.454Z</t>
   </si>
   <si>
     <t>VOL-LOAD-11</t>
@@ -1923,7 +1923,7 @@
     <t>Verify Volunteers screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.114Z</t>
+    <t>2026-07-25T15:58:35.580Z</t>
   </si>
   <si>
     <t>VOL-LOAD-12</t>
@@ -1932,7 +1932,7 @@
     <t>Verify Volunteers screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.143Z</t>
+    <t>2026-07-25T15:58:35.672Z</t>
   </si>
   <si>
     <t>VOL-LOAD-13</t>
@@ -1941,7 +1941,7 @@
     <t>Verify Volunteers screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.171Z</t>
+    <t>2026-07-25T15:58:35.773Z</t>
   </si>
   <si>
     <t>VOL-LOAD-14</t>
@@ -1950,7 +1950,7 @@
     <t>Verify Volunteers screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.198Z</t>
+    <t>2026-07-25T15:58:35.903Z</t>
   </si>
   <si>
     <t>VOL-LOAD-15</t>
@@ -1959,7 +1959,7 @@
     <t>Verify Volunteers screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.227Z</t>
+    <t>2026-07-25T15:58:36.076Z</t>
   </si>
   <si>
     <t>VOL-LOAD-16</t>
@@ -1968,7 +1968,7 @@
     <t>Verify Volunteers screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.254Z</t>
+    <t>2026-07-25T15:58:36.244Z</t>
   </si>
   <si>
     <t>VOL-LOAD-17</t>
@@ -1977,7 +1977,7 @@
     <t>Verify Volunteers screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.284Z</t>
+    <t>2026-07-25T15:58:36.376Z</t>
   </si>
   <si>
     <t>VOL-LOAD-18</t>
@@ -1986,7 +1986,7 @@
     <t>Verify Volunteers screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.311Z</t>
+    <t>2026-07-25T15:58:36.528Z</t>
   </si>
   <si>
     <t>VOL-LOAD-19</t>
@@ -1995,7 +1995,7 @@
     <t>Verify Volunteers screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.339Z</t>
+    <t>2026-07-25T15:58:36.693Z</t>
   </si>
   <si>
     <t>VOL-LOAD-20</t>
@@ -2004,7 +2004,7 @@
     <t>Verify Volunteers screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.368Z</t>
+    <t>2026-07-25T15:58:36.821Z</t>
   </si>
   <si>
     <t>VOL-LOAD-21</t>
@@ -2013,7 +2013,7 @@
     <t>Verify Volunteers screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.399Z</t>
+    <t>2026-07-25T15:58:37.169Z</t>
   </si>
   <si>
     <t>VOL-LOAD-22</t>
@@ -2022,7 +2022,7 @@
     <t>Verify Volunteers screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.429Z</t>
+    <t>2026-07-25T15:58:37.411Z</t>
   </si>
   <si>
     <t>VOL-LOAD-23</t>
@@ -2031,7 +2031,7 @@
     <t>Verify Volunteers screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.457Z</t>
+    <t>2026-07-25T15:58:37.639Z</t>
   </si>
   <si>
     <t>VOL-LOAD-24</t>
@@ -2040,7 +2040,7 @@
     <t>Verify Volunteers screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.486Z</t>
+    <t>2026-07-25T15:58:37.987Z</t>
   </si>
   <si>
     <t>VOL-LOAD-25</t>
@@ -2049,7 +2049,7 @@
     <t>Verify Volunteers screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.517Z</t>
+    <t>2026-07-25T15:58:38.187Z</t>
   </si>
   <si>
     <t>VOL-LOAD-26</t>
@@ -2058,7 +2058,7 @@
     <t>Verify Volunteers screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.551Z</t>
+    <t>2026-07-25T15:58:38.335Z</t>
   </si>
   <si>
     <t>VOL-LOAD-27</t>
@@ -2067,7 +2067,7 @@
     <t>Verify Volunteers screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.581Z</t>
+    <t>2026-07-25T15:58:38.487Z</t>
   </si>
   <si>
     <t>VOL-LOAD-28</t>
@@ -2076,7 +2076,7 @@
     <t>Verify Volunteers screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.609Z</t>
+    <t>2026-07-25T15:58:38.639Z</t>
   </si>
   <si>
     <t>VOL-LOAD-29</t>
@@ -2085,7 +2085,7 @@
     <t>Verify Volunteers screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.638Z</t>
+    <t>2026-07-25T15:58:38.772Z</t>
   </si>
   <si>
     <t>VOL-LOAD-30</t>
@@ -2094,7 +2094,7 @@
     <t>Verify Volunteers screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.666Z</t>
+    <t>2026-07-25T15:58:38.916Z</t>
   </si>
   <si>
     <t>VOL-LOAD-31</t>
@@ -2103,7 +2103,7 @@
     <t>Verify Volunteers screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.694Z</t>
+    <t>2026-07-25T15:58:39.054Z</t>
   </si>
   <si>
     <t>VOL-LOAD-32</t>
@@ -2112,7 +2112,7 @@
     <t>Verify Volunteers screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.727Z</t>
+    <t>2026-07-25T15:58:39.205Z</t>
   </si>
   <si>
     <t>VOL-LOAD-33</t>
@@ -2121,7 +2121,7 @@
     <t>Verify Volunteers screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.771Z</t>
+    <t>2026-07-25T15:58:39.365Z</t>
   </si>
   <si>
     <t>VOL-LOAD-34</t>
@@ -2130,7 +2130,7 @@
     <t>Verify Volunteers screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.805Z</t>
+    <t>2026-07-25T15:58:39.767Z</t>
   </si>
   <si>
     <t>VOL-LOAD-35</t>
@@ -2139,7 +2139,7 @@
     <t>Verify Volunteers screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.843Z</t>
+    <t>2026-07-25T15:58:39.971Z</t>
   </si>
   <si>
     <t>VOL-LOAD-36</t>
@@ -2148,7 +2148,7 @@
     <t>Verify Volunteers screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.873Z</t>
+    <t>2026-07-25T15:58:40.102Z</t>
   </si>
   <si>
     <t>VOL-LOAD-37</t>
@@ -2157,7 +2157,7 @@
     <t>Verify Volunteers screen response speed during Concurrency test (Case #37)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.902Z</t>
+    <t>2026-07-25T15:58:40.231Z</t>
   </si>
   <si>
     <t>EVT-LOAD-01</t>
@@ -2166,7 +2166,7 @@
     <t>Verify Events screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.933Z</t>
+    <t>2026-07-25T15:58:40.354Z</t>
   </si>
   <si>
     <t>EVT-LOAD-02</t>
@@ -2175,7 +2175,7 @@
     <t>Verify Events screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.966Z</t>
+    <t>2026-07-25T15:58:40.482Z</t>
   </si>
   <si>
     <t>EVT-LOAD-03</t>
@@ -2184,7 +2184,7 @@
     <t>Verify Events screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:50.997Z</t>
+    <t>2026-07-25T15:58:40.609Z</t>
   </si>
   <si>
     <t>EVT-LOAD-04</t>
@@ -2193,7 +2193,7 @@
     <t>Verify Events screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.028Z</t>
+    <t>2026-07-25T15:58:40.729Z</t>
   </si>
   <si>
     <t>EVT-LOAD-05</t>
@@ -2202,7 +2202,7 @@
     <t>Verify Events screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.065Z</t>
+    <t>2026-07-25T15:58:40.852Z</t>
   </si>
   <si>
     <t>EVT-LOAD-06</t>
@@ -2211,7 +2211,7 @@
     <t>Verify Events screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.094Z</t>
+    <t>2026-07-25T15:58:40.983Z</t>
   </si>
   <si>
     <t>EVT-LOAD-07</t>
@@ -2220,7 +2220,7 @@
     <t>Verify Events screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.136Z</t>
+    <t>2026-07-25T15:58:41.101Z</t>
   </si>
   <si>
     <t>EVT-LOAD-08</t>
@@ -2229,7 +2229,7 @@
     <t>Verify Events screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.174Z</t>
+    <t>2026-07-25T15:58:41.224Z</t>
   </si>
   <si>
     <t>EVT-LOAD-09</t>
@@ -2238,7 +2238,7 @@
     <t>Verify Events screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.208Z</t>
+    <t>2026-07-25T15:58:41.343Z</t>
   </si>
   <si>
     <t>EVT-LOAD-10</t>
@@ -2247,7 +2247,7 @@
     <t>Verify Events screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.243Z</t>
+    <t>2026-07-25T15:58:41.460Z</t>
   </si>
   <si>
     <t>EVT-LOAD-11</t>
@@ -2256,7 +2256,7 @@
     <t>Verify Events screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.282Z</t>
+    <t>2026-07-25T15:58:41.571Z</t>
   </si>
   <si>
     <t>EVT-LOAD-12</t>
@@ -2265,7 +2265,7 @@
     <t>Verify Events screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.313Z</t>
+    <t>2026-07-25T15:58:41.682Z</t>
   </si>
   <si>
     <t>EVT-LOAD-13</t>
@@ -2274,7 +2274,7 @@
     <t>Verify Events screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.351Z</t>
+    <t>2026-07-25T15:58:41.805Z</t>
   </si>
   <si>
     <t>EVT-LOAD-14</t>
@@ -2283,7 +2283,7 @@
     <t>Verify Events screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.386Z</t>
+    <t>2026-07-25T15:58:41.920Z</t>
   </si>
   <si>
     <t>EVT-LOAD-15</t>
@@ -2292,7 +2292,7 @@
     <t>Verify Events screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.417Z</t>
+    <t>2026-07-25T15:58:42.044Z</t>
   </si>
   <si>
     <t>EVT-LOAD-16</t>
@@ -2301,7 +2301,7 @@
     <t>Verify Events screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.453Z</t>
+    <t>2026-07-25T15:58:42.163Z</t>
   </si>
   <si>
     <t>EVT-LOAD-17</t>
@@ -2310,7 +2310,7 @@
     <t>Verify Events screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.493Z</t>
+    <t>2026-07-25T15:58:42.285Z</t>
   </si>
   <si>
     <t>EVT-LOAD-18</t>
@@ -2319,7 +2319,7 @@
     <t>Verify Events screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.532Z</t>
+    <t>2026-07-25T15:58:42.420Z</t>
   </si>
   <si>
     <t>EVT-LOAD-19</t>
@@ -2328,7 +2328,7 @@
     <t>Verify Events screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.564Z</t>
+    <t>2026-07-25T15:58:42.547Z</t>
   </si>
   <si>
     <t>EVT-LOAD-20</t>
@@ -2337,7 +2337,7 @@
     <t>Verify Events screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.595Z</t>
+    <t>2026-07-25T15:58:42.676Z</t>
   </si>
   <si>
     <t>EVT-LOAD-21</t>
@@ -2346,7 +2346,7 @@
     <t>Verify Events screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.644Z</t>
+    <t>2026-07-25T15:58:42.831Z</t>
   </si>
   <si>
     <t>EVT-LOAD-22</t>
@@ -2355,7 +2355,7 @@
     <t>Verify Events screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.677Z</t>
+    <t>2026-07-25T15:58:42.978Z</t>
   </si>
   <si>
     <t>EVT-LOAD-23</t>
@@ -2364,7 +2364,7 @@
     <t>Verify Events screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.707Z</t>
+    <t>2026-07-25T15:58:43.110Z</t>
   </si>
   <si>
     <t>EVT-LOAD-24</t>
@@ -2373,7 +2373,7 @@
     <t>Verify Events screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.743Z</t>
+    <t>2026-07-25T15:58:43.242Z</t>
   </si>
   <si>
     <t>EVT-LOAD-25</t>
@@ -2382,7 +2382,7 @@
     <t>Verify Events screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.786Z</t>
+    <t>2026-07-25T15:58:43.372Z</t>
   </si>
   <si>
     <t>EVT-LOAD-26</t>
@@ -2391,7 +2391,7 @@
     <t>Verify Events screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.821Z</t>
+    <t>2026-07-25T15:58:43.515Z</t>
   </si>
   <si>
     <t>EVT-LOAD-27</t>
@@ -2400,7 +2400,7 @@
     <t>Verify Events screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.857Z</t>
+    <t>2026-07-25T15:58:43.646Z</t>
   </si>
   <si>
     <t>EVT-LOAD-28</t>
@@ -2409,7 +2409,7 @@
     <t>Verify Events screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.894Z</t>
+    <t>2026-07-25T15:58:43.773Z</t>
   </si>
   <si>
     <t>EVT-LOAD-29</t>
@@ -2418,7 +2418,7 @@
     <t>Verify Events screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.941Z</t>
+    <t>2026-07-25T15:58:43.911Z</t>
   </si>
   <si>
     <t>EVT-LOAD-30</t>
@@ -2427,7 +2427,7 @@
     <t>Verify Events screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:51.993Z</t>
+    <t>2026-07-25T15:58:44.050Z</t>
   </si>
   <si>
     <t>EVT-LOAD-31</t>
@@ -2436,7 +2436,7 @@
     <t>Verify Events screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.039Z</t>
+    <t>2026-07-25T15:58:44.186Z</t>
   </si>
   <si>
     <t>EVT-LOAD-32</t>
@@ -2445,7 +2445,7 @@
     <t>Verify Events screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.084Z</t>
+    <t>2026-07-25T15:58:44.321Z</t>
   </si>
   <si>
     <t>EVT-LOAD-33</t>
@@ -2454,7 +2454,7 @@
     <t>Verify Events screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.122Z</t>
+    <t>2026-07-25T15:58:44.465Z</t>
   </si>
   <si>
     <t>EVT-LOAD-34</t>
@@ -2463,7 +2463,7 @@
     <t>Verify Events screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.170Z</t>
+    <t>2026-07-25T15:58:44.587Z</t>
   </si>
   <si>
     <t>EVT-LOAD-35</t>
@@ -2472,7 +2472,7 @@
     <t>Verify Events screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.216Z</t>
+    <t>2026-07-25T15:58:44.813Z</t>
   </si>
   <si>
     <t>EVT-LOAD-36</t>
@@ -2481,7 +2481,7 @@
     <t>Verify Events screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.261Z</t>
+    <t>2026-07-25T15:58:45.066Z</t>
   </si>
   <si>
     <t>EVT-LOAD-37</t>
@@ -2490,7 +2490,7 @@
     <t>Verify Events screen response speed during Concurrency test (Case #37)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.300Z</t>
+    <t>2026-07-25T15:58:45.361Z</t>
   </si>
   <si>
     <t>ATT-LOAD-01</t>
@@ -2499,7 +2499,7 @@
     <t>Verify Attendance screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.339Z</t>
+    <t>2026-07-25T15:58:45.660Z</t>
   </si>
   <si>
     <t>ATT-LOAD-02</t>
@@ -2508,7 +2508,7 @@
     <t>Verify Attendance screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.379Z</t>
+    <t>2026-07-25T15:58:45.846Z</t>
   </si>
   <si>
     <t>ATT-LOAD-03</t>
@@ -2517,7 +2517,7 @@
     <t>Verify Attendance screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.416Z</t>
+    <t>2026-07-25T15:58:46.032Z</t>
   </si>
   <si>
     <t>ATT-LOAD-04</t>
@@ -2526,7 +2526,7 @@
     <t>Verify Attendance screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.453Z</t>
+    <t>2026-07-25T15:58:46.204Z</t>
   </si>
   <si>
     <t>ATT-LOAD-05</t>
@@ -2535,7 +2535,7 @@
     <t>Verify Attendance screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.502Z</t>
+    <t>2026-07-25T15:58:46.415Z</t>
   </si>
   <si>
     <t>ATT-LOAD-06</t>
@@ -2544,7 +2544,7 @@
     <t>Verify Attendance screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.548Z</t>
+    <t>2026-07-25T15:58:46.610Z</t>
   </si>
   <si>
     <t>ATT-LOAD-07</t>
@@ -2553,7 +2553,7 @@
     <t>Verify Attendance screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.591Z</t>
+    <t>2026-07-25T15:58:46.776Z</t>
   </si>
   <si>
     <t>ATT-LOAD-08</t>
@@ -2562,7 +2562,7 @@
     <t>Verify Attendance screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.637Z</t>
+    <t>2026-07-25T15:58:46.965Z</t>
   </si>
   <si>
     <t>ATT-LOAD-09</t>
@@ -2571,7 +2571,7 @@
     <t>Verify Attendance screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.682Z</t>
+    <t>2026-07-25T15:58:47.174Z</t>
   </si>
   <si>
     <t>ATT-LOAD-10</t>
@@ -2580,7 +2580,7 @@
     <t>Verify Attendance screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.720Z</t>
+    <t>2026-07-25T15:58:47.327Z</t>
   </si>
   <si>
     <t>ATT-LOAD-11</t>
@@ -2589,7 +2589,7 @@
     <t>Verify Attendance screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.757Z</t>
+    <t>2026-07-25T15:58:47.477Z</t>
   </si>
   <si>
     <t>ATT-LOAD-12</t>
@@ -2598,7 +2598,7 @@
     <t>Verify Attendance screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.793Z</t>
+    <t>2026-07-25T15:58:47.636Z</t>
   </si>
   <si>
     <t>ATT-LOAD-13</t>
@@ -2607,7 +2607,7 @@
     <t>Verify Attendance screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.831Z</t>
+    <t>2026-07-25T15:58:47.780Z</t>
   </si>
   <si>
     <t>ATT-LOAD-14</t>
@@ -2616,7 +2616,7 @@
     <t>Verify Attendance screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.865Z</t>
+    <t>2026-07-25T15:58:47.924Z</t>
   </si>
   <si>
     <t>ATT-LOAD-15</t>
@@ -2625,7 +2625,7 @@
     <t>Verify Attendance screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.912Z</t>
+    <t>2026-07-25T15:58:48.073Z</t>
   </si>
   <si>
     <t>ATT-LOAD-16</t>
@@ -2634,7 +2634,7 @@
     <t>Verify Attendance screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:52.959Z</t>
+    <t>2026-07-25T15:58:48.218Z</t>
   </si>
   <si>
     <t>ATT-LOAD-17</t>
@@ -2643,7 +2643,7 @@
     <t>Verify Attendance screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.007Z</t>
+    <t>2026-07-25T15:58:48.316Z</t>
   </si>
   <si>
     <t>ATT-LOAD-18</t>
@@ -2652,7 +2652,7 @@
     <t>Verify Attendance screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.064Z</t>
+    <t>2026-07-25T15:58:48.450Z</t>
   </si>
   <si>
     <t>ATT-LOAD-19</t>
@@ -2661,7 +2661,7 @@
     <t>Verify Attendance screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.103Z</t>
+    <t>2026-07-25T15:58:48.601Z</t>
   </si>
   <si>
     <t>ATT-LOAD-20</t>
@@ -2670,7 +2670,7 @@
     <t>Verify Attendance screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.139Z</t>
+    <t>2026-07-25T15:58:48.740Z</t>
   </si>
   <si>
     <t>ATT-LOAD-21</t>
@@ -2679,7 +2679,7 @@
     <t>Verify Attendance screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.185Z</t>
+    <t>2026-07-25T15:58:48.909Z</t>
   </si>
   <si>
     <t>ATT-LOAD-22</t>
@@ -2688,7 +2688,7 @@
     <t>Verify Attendance screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.223Z</t>
+    <t>2026-07-25T15:58:49.059Z</t>
   </si>
   <si>
     <t>ATT-LOAD-23</t>
@@ -2697,7 +2697,7 @@
     <t>Verify Attendance screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.262Z</t>
+    <t>2026-07-25T15:58:49.212Z</t>
   </si>
   <si>
     <t>ATT-LOAD-24</t>
@@ -2706,7 +2706,7 @@
     <t>Verify Attendance screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.303Z</t>
+    <t>2026-07-25T15:58:49.366Z</t>
   </si>
   <si>
     <t>ATT-LOAD-25</t>
@@ -2715,7 +2715,7 @@
     <t>Verify Attendance screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.341Z</t>
+    <t>2026-07-25T15:58:49.515Z</t>
   </si>
   <si>
     <t>ATT-LOAD-26</t>
@@ -2724,7 +2724,7 @@
     <t>Verify Attendance screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.378Z</t>
+    <t>2026-07-25T15:58:49.671Z</t>
   </si>
   <si>
     <t>ATT-LOAD-27</t>
@@ -2733,7 +2733,7 @@
     <t>Verify Attendance screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.417Z</t>
+    <t>2026-07-25T15:58:49.820Z</t>
   </si>
   <si>
     <t>ATT-LOAD-28</t>
@@ -2742,7 +2742,7 @@
     <t>Verify Attendance screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.459Z</t>
+    <t>2026-07-25T15:58:49.967Z</t>
   </si>
   <si>
     <t>ATT-LOAD-29</t>
@@ -2751,7 +2751,7 @@
     <t>Verify Attendance screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.498Z</t>
+    <t>2026-07-25T15:58:50.119Z</t>
   </si>
   <si>
     <t>ATT-LOAD-30</t>
@@ -2760,7 +2760,7 @@
     <t>Verify Attendance screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.539Z</t>
+    <t>2026-07-25T15:58:50.268Z</t>
   </si>
   <si>
     <t>ATT-LOAD-31</t>
@@ -2769,7 +2769,7 @@
     <t>Verify Attendance screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.583Z</t>
+    <t>2026-07-25T15:58:50.420Z</t>
   </si>
   <si>
     <t>ATT-LOAD-32</t>
@@ -2778,7 +2778,7 @@
     <t>Verify Attendance screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.648Z</t>
+    <t>2026-07-25T15:58:50.761Z</t>
   </si>
   <si>
     <t>ATT-LOAD-33</t>
@@ -2787,7 +2787,7 @@
     <t>Verify Attendance screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.698Z</t>
+    <t>2026-07-25T15:58:51.128Z</t>
   </si>
   <si>
     <t>ATT-LOAD-34</t>
@@ -2796,7 +2796,7 @@
     <t>Verify Attendance screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.742Z</t>
+    <t>2026-07-25T15:58:51.802Z</t>
   </si>
   <si>
     <t>ATT-LOAD-35</t>
@@ -2805,7 +2805,7 @@
     <t>Verify Attendance screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.776Z</t>
+    <t>2026-07-25T15:58:52.160Z</t>
   </si>
   <si>
     <t>ATT-LOAD-36</t>
@@ -2814,7 +2814,7 @@
     <t>Verify Attendance screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.816Z</t>
+    <t>2026-07-25T15:58:52.398Z</t>
   </si>
   <si>
     <t>ATT-LOAD-37</t>
@@ -2823,7 +2823,7 @@
     <t>Verify Attendance screen response speed during Concurrency test (Case #37)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.850Z</t>
+    <t>2026-07-25T15:58:52.600Z</t>
   </si>
   <si>
     <t>REP-LOAD-01</t>
@@ -2832,7 +2832,7 @@
     <t>Verify Reports screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.882Z</t>
+    <t>2026-07-25T15:58:53.109Z</t>
   </si>
   <si>
     <t>REP-LOAD-02</t>
@@ -2841,7 +2841,7 @@
     <t>Verify Reports screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.917Z</t>
+    <t>2026-07-25T15:58:53.406Z</t>
   </si>
   <si>
     <t>REP-LOAD-03</t>
@@ -2850,7 +2850,7 @@
     <t>Verify Reports screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.953Z</t>
+    <t>2026-07-25T15:58:53.561Z</t>
   </si>
   <si>
     <t>REP-LOAD-04</t>
@@ -2859,7 +2859,7 @@
     <t>Verify Reports screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:53.991Z</t>
+    <t>2026-07-25T15:58:53.739Z</t>
   </si>
   <si>
     <t>REP-LOAD-05</t>
@@ -2868,7 +2868,7 @@
     <t>Verify Reports screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.032Z</t>
+    <t>2026-07-25T15:58:53.888Z</t>
   </si>
   <si>
     <t>REP-LOAD-06</t>
@@ -2877,7 +2877,7 @@
     <t>Verify Reports screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.082Z</t>
+    <t>2026-07-25T15:58:54.042Z</t>
   </si>
   <si>
     <t>REP-LOAD-07</t>
@@ -2886,7 +2886,7 @@
     <t>Verify Reports screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.118Z</t>
+    <t>2026-07-25T15:58:54.211Z</t>
   </si>
   <si>
     <t>REP-LOAD-08</t>
@@ -2895,7 +2895,7 @@
     <t>Verify Reports screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.159Z</t>
+    <t>2026-07-25T15:58:54.354Z</t>
   </si>
   <si>
     <t>REP-LOAD-09</t>
@@ -2904,7 +2904,7 @@
     <t>Verify Reports screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.203Z</t>
+    <t>2026-07-25T15:58:54.497Z</t>
   </si>
   <si>
     <t>REP-LOAD-10</t>
@@ -2913,7 +2913,7 @@
     <t>Verify Reports screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.249Z</t>
+    <t>2026-07-25T15:58:54.668Z</t>
   </si>
   <si>
     <t>REP-LOAD-11</t>
@@ -2922,7 +2922,7 @@
     <t>Verify Reports screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.294Z</t>
+    <t>2026-07-25T15:58:54.821Z</t>
   </si>
   <si>
     <t>REP-LOAD-12</t>
@@ -2937,7 +2937,7 @@
     <t>Memory spiked to 720MB (Garbage collection latency)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.334Z</t>
+    <t>2026-07-25T15:58:54.985Z</t>
   </si>
   <si>
     <t>REP-LOAD-13</t>
@@ -2946,7 +2946,7 @@
     <t>Verify Reports screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.386Z</t>
+    <t>2026-07-25T15:58:55.131Z</t>
   </si>
   <si>
     <t>REP-LOAD-14</t>
@@ -2955,7 +2955,7 @@
     <t>Verify Reports screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.424Z</t>
+    <t>2026-07-25T15:58:55.307Z</t>
   </si>
   <si>
     <t>REP-LOAD-15</t>
@@ -2964,7 +2964,7 @@
     <t>Verify Reports screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.469Z</t>
+    <t>2026-07-25T15:58:55.464Z</t>
   </si>
   <si>
     <t>REP-LOAD-16</t>
@@ -2973,7 +2973,7 @@
     <t>Verify Reports screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.512Z</t>
+    <t>2026-07-25T15:58:55.631Z</t>
   </si>
   <si>
     <t>REP-LOAD-17</t>
@@ -2982,7 +2982,7 @@
     <t>Verify Reports screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.567Z</t>
+    <t>2026-07-25T15:58:55.793Z</t>
   </si>
   <si>
     <t>REP-LOAD-18</t>
@@ -2991,7 +2991,7 @@
     <t>Verify Reports screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.612Z</t>
+    <t>2026-07-25T15:58:55.961Z</t>
   </si>
   <si>
     <t>REP-LOAD-19</t>
@@ -3000,7 +3000,7 @@
     <t>Verify Reports screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.649Z</t>
+    <t>2026-07-25T15:58:56.117Z</t>
   </si>
   <si>
     <t>REP-LOAD-20</t>
@@ -3009,7 +3009,7 @@
     <t>Verify Reports screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.687Z</t>
+    <t>2026-07-25T15:58:56.289Z</t>
   </si>
   <si>
     <t>REP-LOAD-21</t>
@@ -3018,7 +3018,7 @@
     <t>Verify Reports screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.728Z</t>
+    <t>2026-07-25T15:58:56.450Z</t>
   </si>
   <si>
     <t>REP-LOAD-22</t>
@@ -3027,7 +3027,7 @@
     <t>Verify Reports screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.768Z</t>
+    <t>2026-07-25T15:58:56.617Z</t>
   </si>
   <si>
     <t>REP-LOAD-23</t>
@@ -3036,7 +3036,7 @@
     <t>Verify Reports screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.823Z</t>
+    <t>2026-07-25T15:58:56.784Z</t>
   </si>
   <si>
     <t>REP-LOAD-24</t>
@@ -3045,7 +3045,7 @@
     <t>Verify Reports screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.862Z</t>
+    <t>2026-07-25T15:58:56.976Z</t>
   </si>
   <si>
     <t>REP-LOAD-25</t>
@@ -3054,7 +3054,7 @@
     <t>Verify Reports screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.901Z</t>
+    <t>2026-07-25T15:58:57.143Z</t>
   </si>
   <si>
     <t>REP-LOAD-26</t>
@@ -3063,7 +3063,7 @@
     <t>Verify Reports screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.943Z</t>
+    <t>2026-07-25T15:58:57.323Z</t>
   </si>
   <si>
     <t>REP-LOAD-27</t>
@@ -3072,7 +3072,7 @@
     <t>Verify Reports screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:54.985Z</t>
+    <t>2026-07-25T15:58:57.493Z</t>
   </si>
   <si>
     <t>REP-LOAD-28</t>
@@ -3081,7 +3081,7 @@
     <t>Verify Reports screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.028Z</t>
+    <t>2026-07-25T15:58:57.664Z</t>
   </si>
   <si>
     <t>REP-LOAD-29</t>
@@ -3090,7 +3090,7 @@
     <t>Verify Reports screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.077Z</t>
+    <t>2026-07-25T15:58:57.835Z</t>
   </si>
   <si>
     <t>REP-LOAD-30</t>
@@ -3099,7 +3099,7 @@
     <t>Verify Reports screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.122Z</t>
+    <t>2026-07-25T15:58:58.129Z</t>
   </si>
   <si>
     <t>REP-LOAD-31</t>
@@ -3108,7 +3108,7 @@
     <t>Verify Reports screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.192Z</t>
+    <t>2026-07-25T15:58:58.440Z</t>
   </si>
   <si>
     <t>REP-LOAD-32</t>
@@ -3117,7 +3117,7 @@
     <t>Verify Reports screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.231Z</t>
+    <t>2026-07-25T15:58:58.797Z</t>
   </si>
   <si>
     <t>REP-LOAD-33</t>
@@ -3126,7 +3126,7 @@
     <t>Verify Reports screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.277Z</t>
+    <t>2026-07-25T15:58:59.014Z</t>
   </si>
   <si>
     <t>REP-LOAD-34</t>
@@ -3135,7 +3135,7 @@
     <t>Verify Reports screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.316Z</t>
+    <t>2026-07-25T15:58:59.230Z</t>
   </si>
   <si>
     <t>REP-LOAD-35</t>
@@ -3144,7 +3144,7 @@
     <t>Verify Reports screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.361Z</t>
+    <t>2026-07-25T15:58:59.445Z</t>
   </si>
   <si>
     <t>REP-LOAD-36</t>
@@ -3153,7 +3153,7 @@
     <t>Verify Reports screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.407Z</t>
+    <t>2026-07-25T15:58:59.661Z</t>
   </si>
   <si>
     <t>REP-LOAD-37</t>
@@ -3162,7 +3162,7 @@
     <t>Verify Reports screen response speed during Concurrency test (Case #37)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.463Z</t>
+    <t>2026-07-25T15:58:59.871Z</t>
   </si>
   <si>
     <t>SET-LOAD-01</t>
@@ -3171,7 +3171,7 @@
     <t>Verify Settings screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.507Z</t>
+    <t>2026-07-25T15:59:00.117Z</t>
   </si>
   <si>
     <t>SET-LOAD-02</t>
@@ -3180,7 +3180,7 @@
     <t>Verify Settings screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.554Z</t>
+    <t>2026-07-25T15:59:00.396Z</t>
   </si>
   <si>
     <t>SET-LOAD-03</t>
@@ -3189,7 +3189,7 @@
     <t>Verify Settings screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.599Z</t>
+    <t>2026-07-25T15:59:00.572Z</t>
   </si>
   <si>
     <t>SET-LOAD-04</t>
@@ -3198,7 +3198,7 @@
     <t>Verify Settings screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.644Z</t>
+    <t>2026-07-25T15:59:00.749Z</t>
   </si>
   <si>
     <t>SET-LOAD-05</t>
@@ -3207,7 +3207,7 @@
     <t>Verify Settings screen response speed during API Gateway test (Case #5)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.686Z</t>
+    <t>2026-07-25T15:59:00.928Z</t>
   </si>
   <si>
     <t>SET-LOAD-06</t>
@@ -3216,7 +3216,7 @@
     <t>Verify Settings screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.730Z</t>
+    <t>2026-07-25T15:59:01.106Z</t>
   </si>
   <si>
     <t>SET-LOAD-07</t>
@@ -3225,7 +3225,7 @@
     <t>Verify Settings screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.776Z</t>
+    <t>2026-07-25T15:59:01.267Z</t>
   </si>
   <si>
     <t>SET-LOAD-08</t>
@@ -3234,7 +3234,7 @@
     <t>Verify Settings screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.826Z</t>
+    <t>2026-07-25T15:59:01.420Z</t>
   </si>
   <si>
     <t>SET-LOAD-09</t>
@@ -3243,7 +3243,7 @@
     <t>Verify Settings screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.870Z</t>
+    <t>2026-07-25T15:59:01.605Z</t>
   </si>
   <si>
     <t>SET-LOAD-10</t>
@@ -3252,7 +3252,7 @@
     <t>Verify Settings screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.913Z</t>
+    <t>2026-07-25T15:59:01.787Z</t>
   </si>
   <si>
     <t>SET-LOAD-11</t>
@@ -3261,7 +3261,7 @@
     <t>Verify Settings screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:55.953Z</t>
+    <t>2026-07-25T15:59:01.960Z</t>
   </si>
   <si>
     <t>SET-LOAD-12</t>
@@ -3270,7 +3270,7 @@
     <t>Verify Settings screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.002Z</t>
+    <t>2026-07-25T15:59:02.126Z</t>
   </si>
   <si>
     <t>SET-LOAD-13</t>
@@ -3279,7 +3279,7 @@
     <t>Verify Settings screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.052Z</t>
+    <t>2026-07-25T15:59:02.297Z</t>
   </si>
   <si>
     <t>SET-LOAD-14</t>
@@ -3288,7 +3288,7 @@
     <t>Verify Settings screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.101Z</t>
+    <t>2026-07-25T15:59:02.458Z</t>
   </si>
   <si>
     <t>SET-LOAD-15</t>
@@ -3297,7 +3297,7 @@
     <t>Verify Settings screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.142Z</t>
+    <t>2026-07-25T15:59:02.634Z</t>
   </si>
   <si>
     <t>SET-LOAD-16</t>
@@ -3306,7 +3306,7 @@
     <t>Verify Settings screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.188Z</t>
+    <t>2026-07-25T15:59:02.807Z</t>
   </si>
   <si>
     <t>SET-LOAD-17</t>
@@ -3315,7 +3315,7 @@
     <t>Verify Settings screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.229Z</t>
+    <t>2026-07-25T15:59:02.978Z</t>
   </si>
   <si>
     <t>SET-LOAD-18</t>
@@ -3324,7 +3324,7 @@
     <t>Verify Settings screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.277Z</t>
+    <t>2026-07-25T15:59:03.155Z</t>
   </si>
   <si>
     <t>SET-LOAD-19</t>
@@ -3333,7 +3333,7 @@
     <t>Verify Settings screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.319Z</t>
+    <t>2026-07-25T15:59:03.344Z</t>
   </si>
   <si>
     <t>SET-LOAD-20</t>
@@ -3342,7 +3342,7 @@
     <t>Verify Settings screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.374Z</t>
+    <t>2026-07-25T15:59:03.519Z</t>
   </si>
   <si>
     <t>SET-LOAD-21</t>
@@ -3351,7 +3351,7 @@
     <t>Verify Settings screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.419Z</t>
+    <t>2026-07-25T15:59:03.817Z</t>
   </si>
   <si>
     <t>SET-LOAD-22</t>
@@ -3360,7 +3360,7 @@
     <t>Verify Settings screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.462Z</t>
+    <t>2026-07-25T15:59:03.998Z</t>
   </si>
   <si>
     <t>SET-LOAD-23</t>
@@ -3369,7 +3369,7 @@
     <t>Verify Settings screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.503Z</t>
+    <t>2026-07-25T15:59:04.355Z</t>
   </si>
   <si>
     <t>SET-LOAD-24</t>
@@ -3378,7 +3378,7 @@
     <t>Verify Settings screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.547Z</t>
+    <t>2026-07-25T15:59:04.646Z</t>
   </si>
   <si>
     <t>SET-LOAD-25</t>
@@ -3387,7 +3387,7 @@
     <t>Verify Settings screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.596Z</t>
+    <t>2026-07-25T15:59:04.932Z</t>
   </si>
   <si>
     <t>SET-LOAD-26</t>
@@ -3396,7 +3396,7 @@
     <t>Verify Settings screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.643Z</t>
+    <t>2026-07-25T15:59:05.168Z</t>
   </si>
   <si>
     <t>SET-LOAD-27</t>
@@ -3405,7 +3405,7 @@
     <t>Verify Settings screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.684Z</t>
+    <t>2026-07-25T15:59:05.494Z</t>
   </si>
   <si>
     <t>SET-LOAD-28</t>
@@ -3414,7 +3414,7 @@
     <t>Verify Settings screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.746Z</t>
+    <t>2026-07-25T15:59:06.269Z</t>
   </si>
   <si>
     <t>SET-LOAD-29</t>
@@ -3423,7 +3423,7 @@
     <t>Verify Settings screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.791Z</t>
+    <t>2026-07-25T15:59:06.520Z</t>
   </si>
   <si>
     <t>SET-LOAD-30</t>
@@ -3432,7 +3432,7 @@
     <t>Verify Settings screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.835Z</t>
+    <t>2026-07-25T15:59:07.408Z</t>
   </si>
   <si>
     <t>SET-LOAD-31</t>
@@ -3441,7 +3441,7 @@
     <t>Verify Settings screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.878Z</t>
+    <t>2026-07-25T15:59:07.699Z</t>
   </si>
   <si>
     <t>SET-LOAD-32</t>
@@ -3450,7 +3450,7 @@
     <t>Verify Settings screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.922Z</t>
+    <t>2026-07-25T15:59:07.912Z</t>
   </si>
   <si>
     <t>SET-LOAD-33</t>
@@ -3459,7 +3459,7 @@
     <t>Verify Settings screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:56.967Z</t>
+    <t>2026-07-25T15:59:08.089Z</t>
   </si>
   <si>
     <t>SET-LOAD-34</t>
@@ -3468,7 +3468,7 @@
     <t>Verify Settings screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.015Z</t>
+    <t>2026-07-25T15:59:08.273Z</t>
   </si>
   <si>
     <t>SET-LOAD-35</t>
@@ -3477,7 +3477,7 @@
     <t>Verify Settings screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.066Z</t>
+    <t>2026-07-25T15:59:08.473Z</t>
   </si>
   <si>
     <t>SET-LOAD-36</t>
@@ -3486,7 +3486,7 @@
     <t>Verify Settings screen response speed during Latency test (Case #36)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.110Z</t>
+    <t>2026-07-25T15:59:08.645Z</t>
   </si>
   <si>
     <t>SET-LOAD-37</t>
@@ -3495,7 +3495,7 @@
     <t>Verify Settings screen response speed during Concurrency test (Case #37)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.157Z</t>
+    <t>2026-07-25T15:59:08.824Z</t>
   </si>
   <si>
     <t>AI-LOAD-01</t>
@@ -3504,7 +3504,7 @@
     <t>Verify AIChat screen response speed during Latency test (Case #1)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.204Z</t>
+    <t>2026-07-25T15:59:08.991Z</t>
   </si>
   <si>
     <t>AI-LOAD-02</t>
@@ -3513,7 +3513,7 @@
     <t>Verify AIChat screen response speed during Concurrency test (Case #2)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.248Z</t>
+    <t>2026-07-25T15:59:09.169Z</t>
   </si>
   <si>
     <t>AI-LOAD-03</t>
@@ -3522,7 +3522,7 @@
     <t>Verify AIChat screen response speed during Stress Load test (Case #3)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.291Z</t>
+    <t>2026-07-25T15:59:09.352Z</t>
   </si>
   <si>
     <t>AI-LOAD-04</t>
@@ -3531,7 +3531,7 @@
     <t>Verify AIChat screen response speed during DB Performance test (Case #4)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.342Z</t>
+    <t>2026-07-25T15:59:09.538Z</t>
   </si>
   <si>
     <t>AI-LOAD-05</t>
@@ -3546,7 +3546,7 @@
     <t>Average latency increased to 4500ms under 50 active chats</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.388Z</t>
+    <t>2026-07-25T15:59:09.724Z</t>
   </si>
   <si>
     <t>AI-LOAD-06</t>
@@ -3555,7 +3555,7 @@
     <t>Verify AIChat screen response speed during Resource Usage test (Case #6)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.433Z</t>
+    <t>2026-07-25T15:59:09.920Z</t>
   </si>
   <si>
     <t>AI-LOAD-07</t>
@@ -3564,7 +3564,7 @@
     <t>Verify AIChat screen response speed during Throughput test (Case #7)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.478Z</t>
+    <t>2026-07-25T15:59:10.113Z</t>
   </si>
   <si>
     <t>AI-LOAD-08</t>
@@ -3573,7 +3573,7 @@
     <t>Verify AIChat screen response speed during Latency test (Case #8)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.531Z</t>
+    <t>2026-07-25T15:59:10.305Z</t>
   </si>
   <si>
     <t>AI-LOAD-09</t>
@@ -3582,7 +3582,7 @@
     <t>Verify AIChat screen response speed during Concurrency test (Case #9)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.600Z</t>
+    <t>2026-07-25T15:59:10.503Z</t>
   </si>
   <si>
     <t>AI-LOAD-10</t>
@@ -3591,7 +3591,7 @@
     <t>Verify AIChat screen response speed during Stress Load test (Case #10)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.653Z</t>
+    <t>2026-07-25T15:59:10.698Z</t>
   </si>
   <si>
     <t>AI-LOAD-11</t>
@@ -3600,7 +3600,7 @@
     <t>Verify AIChat screen response speed during DB Performance test (Case #11)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.706Z</t>
+    <t>2026-07-25T15:59:10.899Z</t>
   </si>
   <si>
     <t>AI-LOAD-12</t>
@@ -3609,7 +3609,7 @@
     <t>Verify AIChat screen response speed during API Gateway test (Case #12)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.765Z</t>
+    <t>2026-07-25T15:59:11.095Z</t>
   </si>
   <si>
     <t>AI-LOAD-13</t>
@@ -3618,7 +3618,7 @@
     <t>Verify AIChat screen response speed during Resource Usage test (Case #13)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.828Z</t>
+    <t>2026-07-25T15:59:11.371Z</t>
   </si>
   <si>
     <t>AI-LOAD-14</t>
@@ -3627,7 +3627,7 @@
     <t>Verify AIChat screen response speed during Throughput test (Case #14)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.873Z</t>
+    <t>2026-07-25T15:59:11.659Z</t>
   </si>
   <si>
     <t>AI-LOAD-15</t>
@@ -3636,7 +3636,7 @@
     <t>Verify AIChat screen response speed during Latency test (Case #15)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.923Z</t>
+    <t>2026-07-25T15:59:12.078Z</t>
   </si>
   <si>
     <t>AI-LOAD-16</t>
@@ -3645,7 +3645,7 @@
     <t>Verify AIChat screen response speed during Concurrency test (Case #16)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:57.971Z</t>
+    <t>2026-07-25T15:59:12.383Z</t>
   </si>
   <si>
     <t>AI-LOAD-17</t>
@@ -3654,7 +3654,7 @@
     <t>Verify AIChat screen response speed during Stress Load test (Case #17)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.015Z</t>
+    <t>2026-07-25T15:59:12.621Z</t>
   </si>
   <si>
     <t>AI-LOAD-18</t>
@@ -3663,7 +3663,7 @@
     <t>Verify AIChat screen response speed during DB Performance test (Case #18)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.085Z</t>
+    <t>2026-07-25T15:59:12.844Z</t>
   </si>
   <si>
     <t>AI-LOAD-19</t>
@@ -3672,7 +3672,7 @@
     <t>Verify AIChat screen response speed during API Gateway test (Case #19)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.128Z</t>
+    <t>2026-07-25T15:59:13.353Z</t>
   </si>
   <si>
     <t>AI-LOAD-20</t>
@@ -3681,7 +3681,7 @@
     <t>Verify AIChat screen response speed during Resource Usage test (Case #20)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.172Z</t>
+    <t>2026-07-25T15:59:13.894Z</t>
   </si>
   <si>
     <t>AI-LOAD-21</t>
@@ -3690,7 +3690,7 @@
     <t>Verify AIChat screen response speed during Throughput test (Case #21)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.217Z</t>
+    <t>2026-07-25T15:59:14.267Z</t>
   </si>
   <si>
     <t>AI-LOAD-22</t>
@@ -3699,7 +3699,7 @@
     <t>Verify AIChat screen response speed during Latency test (Case #22)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.265Z</t>
+    <t>2026-07-25T15:59:14.523Z</t>
   </si>
   <si>
     <t>AI-LOAD-23</t>
@@ -3708,7 +3708,7 @@
     <t>Verify AIChat screen response speed during Concurrency test (Case #23)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.319Z</t>
+    <t>2026-07-25T15:59:14.717Z</t>
   </si>
   <si>
     <t>AI-LOAD-24</t>
@@ -3717,7 +3717,7 @@
     <t>Verify AIChat screen response speed during Stress Load test (Case #24)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.380Z</t>
+    <t>2026-07-25T15:59:14.922Z</t>
   </si>
   <si>
     <t>AI-LOAD-25</t>
@@ -3726,7 +3726,7 @@
     <t>Verify AIChat screen response speed during DB Performance test (Case #25)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.431Z</t>
+    <t>2026-07-25T15:59:15.125Z</t>
   </si>
   <si>
     <t>AI-LOAD-26</t>
@@ -3735,7 +3735,7 @@
     <t>Verify AIChat screen response speed during API Gateway test (Case #26)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.484Z</t>
+    <t>2026-07-25T15:59:15.327Z</t>
   </si>
   <si>
     <t>AI-LOAD-27</t>
@@ -3744,7 +3744,7 @@
     <t>Verify AIChat screen response speed during Resource Usage test (Case #27)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.538Z</t>
+    <t>2026-07-25T15:59:15.526Z</t>
   </si>
   <si>
     <t>AI-LOAD-28</t>
@@ -3753,7 +3753,7 @@
     <t>Verify AIChat screen response speed during Throughput test (Case #28)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.592Z</t>
+    <t>2026-07-25T15:59:15.731Z</t>
   </si>
   <si>
     <t>AI-LOAD-29</t>
@@ -3762,7 +3762,7 @@
     <t>Verify AIChat screen response speed during Latency test (Case #29)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.663Z</t>
+    <t>2026-07-25T15:59:15.935Z</t>
   </si>
   <si>
     <t>AI-LOAD-30</t>
@@ -3771,7 +3771,7 @@
     <t>Verify AIChat screen response speed during Concurrency test (Case #30)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.716Z</t>
+    <t>2026-07-25T15:59:16.117Z</t>
   </si>
   <si>
     <t>AI-LOAD-31</t>
@@ -3780,7 +3780,7 @@
     <t>Verify AIChat screen response speed during Stress Load test (Case #31)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.764Z</t>
+    <t>2026-07-25T15:59:16.300Z</t>
   </si>
   <si>
     <t>AI-LOAD-32</t>
@@ -3789,7 +3789,7 @@
     <t>Verify AIChat screen response speed during DB Performance test (Case #32)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.812Z</t>
+    <t>2026-07-25T15:59:16.495Z</t>
   </si>
   <si>
     <t>AI-LOAD-33</t>
@@ -3798,7 +3798,7 @@
     <t>Verify AIChat screen response speed during API Gateway test (Case #33)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.875Z</t>
+    <t>2026-07-25T15:59:16.703Z</t>
   </si>
   <si>
     <t>AI-LOAD-34</t>
@@ -3807,7 +3807,7 @@
     <t>Verify AIChat screen response speed during Resource Usage test (Case #34)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:58.945Z</t>
+    <t>2026-07-25T15:59:16.901Z</t>
   </si>
   <si>
     <t>AI-LOAD-35</t>
@@ -3816,7 +3816,7 @@
     <t>Verify AIChat screen response speed during Throughput test (Case #35)</t>
   </si>
   <si>
-    <t>2026-07-23T05:08:59.010Z</t>
+    <t>2026-07-25T15:59:17.117Z</t>
   </si>
 </sst>
 </file>

</xml_diff>